<commit_message>
Auto-atualização RTA - 19/10/2026 16:47
</commit_message>
<xml_diff>
--- a/downloads/RTA_Unidade.xlsx
+++ b/downloads/RTA_Unidade.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M267"/>
+  <dimension ref="A1:M268"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5245,17 +5245,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>RTA-000652</t>
+          <t>RTA-000654</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Rubens Fernandes Junior</t>
+          <t>Jose Carlos Da Silva Gordilho</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Paulo Henrique Pongetti</t>
+          <t>Fabio Machado Fazolin</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -5265,17 +5265,17 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Turno C</t>
+          <t>Turno A</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>04:00:00</t>
+          <t>08:00:00</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>COA</t>
+          <t>Industria Clementina</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -5286,12 +5286,12 @@
       <c r="I83" t="inlineStr"/>
       <c r="J83" t="inlineStr">
         <is>
-          <t>Não houve</t>
+          <t>organizar campanha de fervura de soda na evaporação e inicio de fervura de água nos vácuos</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>1 dia fora da meta com 4 horas seguidas fora da meta</t>
+          <t>fechamento dois dias abaixo da meta</t>
         </is>
       </c>
       <c r="L83" t="inlineStr"/>
@@ -17089,6 +17089,69 @@
         </is>
       </c>
     </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>RTA-000652</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Rubens Fernandes Junior</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>Paulo Henrique Pongetti</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>Turno C</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>04:00:00</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>COA</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I268" t="inlineStr"/>
+      <c r="J268" t="inlineStr">
+        <is>
+          <t>Não houve</t>
+        </is>
+      </c>
+      <c r="K268" t="inlineStr">
+        <is>
+          <t>1 dia fora da meta com 4 horas seguidas fora da meta</t>
+        </is>
+      </c>
+      <c r="L268" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="M268" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto-atualização RTA - 28/10/2026 16:26
</commit_message>
<xml_diff>
--- a/downloads/RTA_Unidade.xlsx
+++ b/downloads/RTA_Unidade.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N280"/>
+  <dimension ref="A1:N281"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5311,27 +5311,27 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>sas:bsc:initiative:4729</t>
+          <t>sas:bsc:initiative:4743</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>RTA-000654</t>
+          <t>RTA-000655</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Jose Carlos Da Silva Gordilho</t>
+          <t>Guilherme Natan da Silva Guandalim</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Fabio Machado Fazolin</t>
+          <t>Angela Cristyna Farias Goncalves</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -5346,23 +5346,19 @@
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Industria Clementina</t>
+          <t>Manutenção Automotiva</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>RNC</t>
         </is>
       </c>
       <c r="J76" t="inlineStr"/>
-      <c r="K76" t="inlineStr">
-        <is>
-          <t>organizar campanha de fervura de soda na evaporação e inicio de fervura de água nos vácuos</t>
-        </is>
-      </c>
+      <c r="K76" t="inlineStr"/>
       <c r="L76" t="inlineStr">
         <is>
-          <t>fechamento dois dias abaixo da meta</t>
+          <t>Pino da mesa do giro CH570</t>
         </is>
       </c>
       <c r="M76" t="inlineStr"/>
@@ -5375,17 +5371,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>sas:bsc:initiative:4743</t>
+          <t>sas:bsc:initiative:4744</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>RTA-000655</t>
+          <t>RTA-000656</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Guilherme Natan da Silva Guandalim</t>
+          <t>Jose Matheus Viana Xavier</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -5395,7 +5391,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -5405,7 +5401,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>08:00:00</t>
+          <t>08:35:00</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -5422,7 +5418,7 @@
       <c r="K77" t="inlineStr"/>
       <c r="L77" t="inlineStr">
         <is>
-          <t>Pino da mesa do giro CH570</t>
+          <t>4002550 - MANGUEIRA HIDRÁULICA JDEERE CB01453671</t>
         </is>
       </c>
       <c r="M77" t="inlineStr"/>
@@ -5435,17 +5431,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>sas:bsc:initiative:4744</t>
+          <t>sas:bsc:initiative:4746</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>RTA-000656</t>
+          <t>RTA-000657</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Jose Matheus Viana Xavier</t>
+          <t>Hugo Henrique Lima da Silva</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -5455,17 +5451,17 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Turno A</t>
+          <t>Turno B</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>08:35:00</t>
+          <t>14:38:00</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -5482,7 +5478,7 @@
       <c r="K78" t="inlineStr"/>
       <c r="L78" t="inlineStr">
         <is>
-          <t>4002550 - MANGUEIRA HIDRÁULICA JDEERE CB01453671</t>
+          <t>coxim do mancal do rolo da ch570</t>
         </is>
       </c>
       <c r="M78" t="inlineStr"/>
@@ -5495,17 +5491,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>sas:bsc:initiative:4746</t>
+          <t>sas:bsc:initiative:4747</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>RTA-000657</t>
+          <t>RTA-000658</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Hugo Henrique Lima da Silva</t>
+          <t>Gilberto Gil Chaves</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -5515,17 +5511,17 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Turno B</t>
+          <t>Turno A</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>14:38:00</t>
+          <t>09:41:00</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -5535,14 +5531,14 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>RNC</t>
+          <t>BOLETIM</t>
         </is>
       </c>
       <c r="J79" t="inlineStr"/>
       <c r="K79" t="inlineStr"/>
       <c r="L79" t="inlineStr">
         <is>
-          <t>coxim do mancal do rolo da ch570</t>
+          <t>partes quentes 6110J</t>
         </is>
       </c>
       <c r="M79" t="inlineStr"/>
@@ -5555,17 +5551,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>sas:bsc:initiative:4747</t>
+          <t>sas:bsc:initiative:4748</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>RTA-000658</t>
+          <t>RTA-000659</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Gilberto Gil Chaves</t>
+          <t>Angela Cristyna Farias Goncalves</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -5575,7 +5571,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -5585,7 +5581,7 @@
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>09:41:00</t>
+          <t>14:36:00</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -5595,14 +5591,14 @@
       </c>
       <c r="I80" t="inlineStr">
         <is>
-          <t>BOLETIM</t>
+          <t>RAF</t>
         </is>
       </c>
       <c r="J80" t="inlineStr"/>
       <c r="K80" t="inlineStr"/>
       <c r="L80" t="inlineStr">
         <is>
-          <t>partes quentes 6110J</t>
+          <t>25110 - EMBREAGEM</t>
         </is>
       </c>
       <c r="M80" t="inlineStr"/>
@@ -5615,12 +5611,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>sas:bsc:initiative:4748</t>
+          <t>sas:bsc:initiative:4749</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>RTA-000659</t>
+          <t>RTA-000660</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -5662,7 +5658,7 @@
       <c r="K81" t="inlineStr"/>
       <c r="L81" t="inlineStr">
         <is>
-          <t>25110 - EMBREAGEM</t>
+          <t>32041 - transmissão</t>
         </is>
       </c>
       <c r="M81" t="inlineStr"/>
@@ -5675,27 +5671,27 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>sas:bsc:initiative:4749</t>
+          <t>sas:bsc:initiative:4750</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>RTA-000660</t>
+          <t>RTA-000661</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
+          <t>Gilberto Gil Chaves</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
           <t>Angela Cristyna Farias Goncalves</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>Angela Cristyna Farias Goncalves</t>
-        </is>
-      </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -5705,7 +5701,7 @@
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>14:36:00</t>
+          <t>09:32:00</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -5715,14 +5711,14 @@
       </c>
       <c r="I82" t="inlineStr">
         <is>
-          <t>RAF</t>
+          <t>RNC</t>
         </is>
       </c>
       <c r="J82" t="inlineStr"/>
       <c r="K82" t="inlineStr"/>
       <c r="L82" t="inlineStr">
         <is>
-          <t>32041 - transmissão</t>
+          <t>campana do transbordo antoniosi</t>
         </is>
       </c>
       <c r="M82" t="inlineStr"/>
@@ -5735,17 +5731,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>sas:bsc:initiative:4750</t>
+          <t>sas:bsc:initiative:4751</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>RTA-000661</t>
+          <t>RTA-000662</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Gilberto Gil Chaves</t>
+          <t>Guilherme Natan da Silva Guandalim</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -5755,7 +5751,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -5765,7 +5761,7 @@
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>09:32:00</t>
+          <t>08:09:00</t>
         </is>
       </c>
       <c r="H83" t="inlineStr">
@@ -5782,7 +5778,7 @@
       <c r="K83" t="inlineStr"/>
       <c r="L83" t="inlineStr">
         <is>
-          <t>campana do transbordo antoniosi</t>
+          <t>cabo flexível do grunner</t>
         </is>
       </c>
       <c r="M83" t="inlineStr"/>
@@ -5795,17 +5791,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>sas:bsc:initiative:4751</t>
+          <t>sas:bsc:initiative:4753</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>RTA-000662</t>
+          <t>RTA-000663</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Guilherme Natan da Silva Guandalim</t>
+          <t>Jose Matheus Viana Xavier</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -5815,7 +5811,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -5825,7 +5821,7 @@
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>08:09:00</t>
+          <t>13:21:00</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
@@ -5842,7 +5838,7 @@
       <c r="K84" t="inlineStr"/>
       <c r="L84" t="inlineStr">
         <is>
-          <t>cabo flexível do grunner</t>
+          <t>eixo do elevador da colhedora - 4002574</t>
         </is>
       </c>
       <c r="M84" t="inlineStr"/>
@@ -5855,54 +5851,58 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>sas:bsc:initiative:4753</t>
+          <t>sas:bsc:initiative:4755</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>RTA-000663</t>
+          <t>RTA-000664</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Jose Matheus Viana Xavier</t>
+          <t>Tarcisio Viana</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Angela Cristyna Farias Goncalves</t>
+          <t>Cesar Antonio Bibiani</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Turno A</t>
+          <t>ADM</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>13:21:00</t>
+          <t>13:34:00</t>
         </is>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>Manutenção Automotiva</t>
+          <t>Planejamento e Controle</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>RNC</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J85" t="inlineStr"/>
-      <c r="K85" t="inlineStr"/>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>Comunicação da Aderência do Indicador Adubação Vinhaça Localizada</t>
+        </is>
+      </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>eixo do elevador da colhedora - 4002574</t>
+          <t>Duas semanas ficando fora da aderência de Lead Time na Adubação Vinhaça Localizada</t>
         </is>
       </c>
       <c r="M85" t="inlineStr"/>
@@ -5915,12 +5915,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>sas:bsc:initiative:4755</t>
+          <t>sas:bsc:initiative:4756</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>RTA-000664</t>
+          <t>RTA-000665</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -5945,7 +5945,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>13:34:00</t>
+          <t>14:09:00</t>
         </is>
       </c>
       <c r="H86" t="inlineStr">
@@ -5961,12 +5961,12 @@
       <c r="J86" t="inlineStr"/>
       <c r="K86" t="inlineStr">
         <is>
-          <t>Comunicação da Aderência do Indicador Adubação Vinhaça Localizada</t>
+          <t>Comunicação da Aderência da Adubação Liquida</t>
         </is>
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>Duas semanas ficando fora da aderência de Lead Time na Adubação Vinhaça Localizada</t>
+          <t>Duas semanas ficando fora da aderência de Lead Time na Adubação Liquida</t>
         </is>
       </c>
       <c r="M86" t="inlineStr"/>
@@ -5979,61 +5979,65 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>sas:bsc:initiative:4756</t>
+          <t>sas:bsc:initiative:4767</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>RTA-000665</t>
+          <t>RTA-000668</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Tarcisio Viana</t>
+          <t>Claudio dos Santos Matos Junior</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Cesar Antonio Bibiani</t>
+          <t>Tiago Jose do Carmo</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>ADM</t>
+          <t>Turno B</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>14:09:00</t>
+          <t>18:57:00</t>
         </is>
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Planejamento e Controle</t>
+          <t>Manutenção Industrial</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Análise de Falha</t>
         </is>
       </c>
       <c r="J87" t="inlineStr"/>
       <c r="K87" t="inlineStr">
         <is>
-          <t>Comunicação da Aderência da Adubação Liquida</t>
+          <t>Parada da caldeira 05 e iniciado procedimento de partida com caldeira 03 e 04.</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>Duas semanas ficando fora da aderência de Lead Time na Adubação Liquida</t>
-        </is>
-      </c>
-      <c r="M87" t="inlineStr"/>
+          <t>Custo acima de 50mil</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>Solicitar Ajuste</t>
+        </is>
+      </c>
       <c r="N87" t="inlineStr">
         <is>
           <t>.</t>
@@ -6043,12 +6047,12 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>sas:bsc:initiative:4767</t>
+          <t>sas:bsc:initiative:4769</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>RTA-000668</t>
+          <t>RTA-000669</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -6063,7 +6067,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -6073,7 +6077,7 @@
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>18:57:00</t>
+          <t>22:00:00</t>
         </is>
       </c>
       <c r="H88" t="inlineStr">
@@ -6089,12 +6093,12 @@
       <c r="J88" t="inlineStr"/>
       <c r="K88" t="inlineStr">
         <is>
-          <t>Parada da caldeira 05 e iniciado procedimento de partida com caldeira 03 e 04.</t>
+          <t>Parada do equipamento para inspeção interna.</t>
         </is>
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>Custo acima de 50mil</t>
+          <t>Parada de Moagem acima de 2h</t>
         </is>
       </c>
       <c r="M88" t="inlineStr">
@@ -6111,12 +6115,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>sas:bsc:initiative:4769</t>
+          <t>sas:bsc:initiative:4771</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>RTA-000669</t>
+          <t>RTA-000670</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -6126,12 +6130,12 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Tiago Jose do Carmo</t>
+          <t>Bruno Gines</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -6141,7 +6145,7 @@
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>22:00:00</t>
+          <t>21:07:00</t>
         </is>
       </c>
       <c r="H89" t="inlineStr">
@@ -6157,7 +6161,7 @@
       <c r="J89" t="inlineStr"/>
       <c r="K89" t="inlineStr">
         <is>
-          <t>Parada do equipamento para inspeção interna.</t>
+          <t>Parada da moenda para retirada de acumulo de bagaço e troca do suporte do pente</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">
@@ -6165,11 +6169,7 @@
           <t>Parada de Moagem acima de 2h</t>
         </is>
       </c>
-      <c r="M89" t="inlineStr">
-        <is>
-          <t>Solicitar Ajuste</t>
-        </is>
-      </c>
+      <c r="M89" t="inlineStr"/>
       <c r="N89" t="inlineStr">
         <is>
           <t>.</t>
@@ -6179,37 +6179,37 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>sas:bsc:initiative:4771</t>
+          <t>sas:bsc:initiative:4799</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>RTA-000670</t>
+          <t>RTA-000671</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Claudio dos Santos Matos Junior</t>
+          <t>Rodrigo Rodrigues De Nazareth Neves</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Bruno Gines</t>
+          <t>Tiago Jose do Carmo</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Turno B</t>
+          <t>Turno A</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>21:07:00</t>
+          <t>09:02:00</t>
         </is>
       </c>
       <c r="H90" t="inlineStr">
@@ -6225,12 +6225,12 @@
       <c r="J90" t="inlineStr"/>
       <c r="K90" t="inlineStr">
         <is>
-          <t>Parada da moenda para retirada de acumulo de bagaço e troca do suporte do pente</t>
+          <t>Reposicionado chapa direcionadora de açucar e soldado a Viga trincada no final da bica</t>
         </is>
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>Parada de Moagem acima de 2h</t>
+          <t>Interrupção do processo por 2:48 horas em função de manutenção mecânica na bica de Jogo</t>
         </is>
       </c>
       <c r="M90" t="inlineStr"/>
@@ -6243,27 +6243,27 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>sas:bsc:initiative:4799</t>
+          <t>sas:bsc:initiative:4862</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>RTA-000671</t>
+          <t>RTA-000673</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Rodrigo Rodrigues De Nazareth Neves</t>
+          <t>Fabio Machado Fazolin</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Tiago Jose do Carmo</t>
+          <t>Kleber Mesquita Caldas</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -6273,28 +6273,28 @@
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>09:02:00</t>
+          <t>08:00:00</t>
         </is>
       </c>
       <c r="H91" t="inlineStr">
         <is>
-          <t>Manutenção Industrial</t>
+          <t>Industria Clementina</t>
         </is>
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>Análise de Falha</t>
+          <t>-</t>
         </is>
       </c>
       <c r="J91" t="inlineStr"/>
       <c r="K91" t="inlineStr">
         <is>
-          <t>Reposicionado chapa direcionadora de açucar e soldado a Viga trincada no final da bica</t>
+          <t>Redução de moagem para controle de níveis do processo</t>
         </is>
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>Interrupção do processo por 2:48 horas em função de manutenção mecânica na bica de Jogo</t>
+          <t>Fechamento com dois dias seguidos fora da meta</t>
         </is>
       </c>
       <c r="M91" t="inlineStr"/>
@@ -19352,6 +19352,74 @@
         </is>
       </c>
     </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>sas:bsc:initiative:4729</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>RTA-000654</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Jose Carlos Da Silva Gordilho</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>Fabio Machado Fazolin</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>Turno A</t>
+        </is>
+      </c>
+      <c r="G281" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="H281" t="inlineStr">
+        <is>
+          <t>Industria Clementina</t>
+        </is>
+      </c>
+      <c r="I281" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J281" t="inlineStr"/>
+      <c r="K281" t="inlineStr">
+        <is>
+          <t>organizar campanha de fervura de soda na evaporação e inicio de fervura de água nos vácuos</t>
+        </is>
+      </c>
+      <c r="L281" t="inlineStr">
+        <is>
+          <t>fechamento dois dias abaixo da meta</t>
+        </is>
+      </c>
+      <c r="M281" t="inlineStr">
+        <is>
+          <t>Aprovado</t>
+        </is>
+      </c>
+      <c r="N281" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>